<commit_message>
Se añaden y se mejora el gnerador del pdf
</commit_message>
<xml_diff>
--- a/config/config.xlsx
+++ b/config/config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ingen\Desktop\Repositorios\AUTO_BATCH_RECORD\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9961CBC4-7DF7-4863-B16E-684CA21FBA06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{616A096B-4DE4-4541-ADCF-283E9DD38E67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -588,7 +588,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -597,7 +597,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>

</xml_diff>